<commit_message>
BDT Account Invoice Name and Description Fix
</commit_message>
<xml_diff>
--- a/Excel/Cash_Management_Entry.xlsx
+++ b/Excel/Cash_Management_Entry.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RPA\Desktop\AccountsPayableProd_Citi\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emon\Documents\UiPath\AccountsPayableProd\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33109286-C67F-4868-8E13-E8F358470096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12056502-949E-4B46-B9BA-63E51D916631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="1620" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CITI" sheetId="2" r:id="rId1"/>
@@ -21,9 +21,6 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -136,9 +133,6 @@
     <t>ENDORSEMENT FEE</t>
   </si>
   <si>
-    <t>STAMP CHARGES COLLECTED</t>
-  </si>
-  <si>
     <t>NOC ISSUANCE CHARGE</t>
   </si>
   <si>
@@ -200,13 +194,16 @@
   </si>
   <si>
     <t>CASH INCENTIVE FILE PROCESSING FEE</t>
+  </si>
+  <si>
+    <t>STAMP CHARGE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -238,29 +235,17 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -324,21 +309,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -348,8 +331,7 @@
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Bad" xfId="1" builtinId="27"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -628,17 +610,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D164EB4A-F712-4130-BEBA-AF20C37CF082}">
-  <dimension ref="A1:F27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F26"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="31.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="40.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.21875" customWidth="1"/>
-    <col min="4" max="4" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1796875" customWidth="1"/>
+    <col min="4" max="4" width="23.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
@@ -658,7 +640,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>32</v>
       </c>
@@ -675,7 +657,7 @@
         <v>27201020010</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>33</v>
       </c>
@@ -692,7 +674,7 @@
         <v>27201020010</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -709,7 +691,7 @@
         <v>27201020010</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -723,8 +705,8 @@
         <v>45101010013</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="8" t="s">
         <v>34</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -743,9 +725,9 @@
         <v>41101096008</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
-        <v>35</v>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="8" t="s">
+        <v>56</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>12</v>
@@ -763,9 +745,9 @@
         <v>41101096008</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
-        <v>36</v>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="6" t="s">
+        <v>35</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>12</v>
@@ -777,24 +759,24 @@
         <v>45101010013</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9">
+        <v>45101010013</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9">
-        <v>45101010013</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
-        <v>45</v>
-      </c>
       <c r="B10" s="3" t="s">
         <v>12</v>
       </c>
@@ -805,9 +787,9 @@
         <v>45101010013</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="10" t="s">
-        <v>54</v>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="9" t="s">
+        <v>53</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>12</v>
@@ -819,9 +801,9 @@
         <v>45101010013</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
-        <v>38</v>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="6" t="s">
+        <v>37</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>12</v>
@@ -833,9 +815,9 @@
         <v>45101010014</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
-        <v>39</v>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="6" t="s">
+        <v>38</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>12</v>
@@ -847,9 +829,9 @@
         <v>45101010014</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
-        <v>46</v>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="6" t="s">
+        <v>45</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>12</v>
@@ -861,9 +843,9 @@
         <v>45101010014</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
-        <v>56</v>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" s="6" t="s">
+        <v>55</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>12</v>
@@ -875,9 +857,9 @@
         <v>45101010014</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="7" t="s">
-        <v>51</v>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" s="6" t="s">
+        <v>50</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>12</v>
@@ -889,9 +871,9 @@
         <v>45101010004</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
-        <v>37</v>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" s="6" t="s">
+        <v>36</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>12</v>
@@ -903,9 +885,9 @@
         <v>45101010004</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
-        <v>47</v>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="6" t="s">
+        <v>46</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>12</v>
@@ -917,9 +899,9 @@
         <v>45101010004</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="7" t="s">
-        <v>48</v>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" s="6" t="s">
+        <v>47</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>12</v>
@@ -931,9 +913,9 @@
         <v>45101010004</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
-        <v>40</v>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" s="6" t="s">
+        <v>39</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>12</v>
@@ -945,9 +927,9 @@
         <v>45101010004</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="7" t="s">
-        <v>49</v>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="6" t="s">
+        <v>48</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>12</v>
@@ -959,9 +941,9 @@
         <v>45101010004</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="11" t="s">
-        <v>55</v>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="10" t="s">
+        <v>54</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>12</v>
@@ -973,9 +955,9 @@
         <v>45101010004</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
-        <v>50</v>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="6" t="s">
+        <v>49</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>12</v>
@@ -987,9 +969,9 @@
         <v>45101010004</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="6" t="s">
-        <v>52</v>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>12</v>
@@ -1001,9 +983,9 @@
         <v>45101010004</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>12</v>
@@ -1015,23 +997,20 @@
         <v>45101010004</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
+        <v>40</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B26" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D26" s="12">
+      <c r="D26" s="11">
         <v>15303010001</v>
       </c>
-      <c r="E26" s="13"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="5"/>
+      <c r="E26" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1045,16 +1024,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C535B3F7-9CCF-4C51-A335-606E16E1CF41}">
   <dimension ref="A1:F14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="29.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="40.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.21875" customWidth="1"/>
-    <col min="4" max="4" width="26.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1796875" customWidth="1"/>
+    <col min="4" max="4" width="26.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1074,7 +1053,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1091,7 +1070,7 @@
         <v>27201020010</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1108,7 +1087,7 @@
         <v>27201020010</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1125,7 +1104,7 @@
         <v>27201020010</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1142,7 +1121,7 @@
         <v>27201020010</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -1162,7 +1141,7 @@
         <v>41101096008</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -1176,7 +1155,7 @@
         <v>45101010013</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
@@ -1196,7 +1175,7 @@
         <v>41101096008</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>15</v>
       </c>
@@ -1216,7 +1195,7 @@
         <v>41101096008</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1236,7 +1215,7 @@
         <v>41101096008</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -1256,7 +1235,7 @@
         <v>41101096008</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -1270,7 +1249,7 @@
         <v>45101010013</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -1290,7 +1269,7 @@
         <v>45101010011</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
CITI Advise submit for approval
</commit_message>
<xml_diff>
--- a/Excel/Cash_Management_Entry.xlsx
+++ b/Excel/Cash_Management_Entry.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Emon\Documents\UiPath\AccountsPayableProd\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12056502-949E-4B46-B9BA-63E51D916631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE92315F-64A0-43CD-A938-D355A7BAD9F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="1620" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -154,9 +154,6 @@
     <t>Prepayment</t>
   </si>
   <si>
-    <t>Accessories/Fabrics/Spare Pars</t>
-  </si>
-  <si>
     <t xml:space="preserve">CREDIT RPT CRG </t>
   </si>
   <si>
@@ -197,6 +194,9 @@
   </si>
   <si>
     <t>STAMP CHARGE</t>
+  </si>
+  <si>
+    <t>TT</t>
   </si>
 </sst>
 </file>
@@ -642,24 +642,21 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E2">
-        <v>15303010001</v>
-      </c>
-      <c r="F2">
-        <v>27201020010</v>
+        <v>12</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2">
+        <v>45101010013</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>7</v>
@@ -676,7 +673,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>7</v>
@@ -693,16 +690,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5">
-        <v>45101010013</v>
+        <v>7</v>
+      </c>
+      <c r="D5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5">
+        <v>15303010001</v>
+      </c>
+      <c r="F5">
+        <v>27201020010</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
@@ -727,7 +727,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>12</v>
@@ -761,7 +761,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>12</v>
@@ -775,7 +775,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>12</v>
@@ -789,7 +789,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>12</v>
@@ -831,7 +831,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>12</v>
@@ -845,7 +845,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>12</v>
@@ -859,7 +859,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>12</v>
@@ -887,7 +887,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>12</v>
@@ -901,7 +901,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>12</v>
@@ -929,7 +929,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>12</v>
@@ -943,7 +943,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>12</v>
@@ -957,7 +957,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>12</v>
@@ -971,7 +971,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>12</v>
@@ -985,7 +985,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>12</v>
@@ -1002,7 +1002,7 @@
         <v>40</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>41</v>

</xml_diff>

<commit_message>
Oracle UI automation: Apply request/check/download, GL download, folders; bank reader updates
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Excel/Cash_Management_Entry.xlsx
+++ b/Excel/Cash_Management_Entry.xlsx
@@ -17,6 +17,7 @@
     <sheet name="CITI_Rules" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="HSBC_Rules" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="DB_Rules" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="CITI_Units" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'SCB_Rules'!$A$1:$E$59</definedName>
@@ -2982,7 +2983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4731,15 +4732,19 @@
           <t>LC_Number_Regex</t>
         </is>
       </c>
-      <c r="C65" s="4" t="n"/>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>^(1418\d{8,9}|\d{3}CTCF\d{9})$</t>
+        </is>
+      </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>later</t>
+          <t>Advice_pdf</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Statement references that are real LC numbers (regex, any case). Blank = any non-empty LC_NUMBER. HSBC: OAA, OAR (OARBD...), DC, DP; NONREF and other references are not looked up</t>
+          <t>Real Dhaka Bank LC number: 1418 + 8 or 9 digits (12 or 13 digits, no B01/G01 suffix, no dot), or the CTCF form such as 202CTCF170730026</t>
         </is>
       </c>
     </row>
@@ -5063,8 +5068,275 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>ADVICE_TEXT</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>LC_Statement_Regex</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>(?&lt;![A-Za-z0-9])(1418\d{8,9}|\d{3}CTCF\d{9})(?:[BG]\d{2})?(?![A-Za-z0-9])</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Bank_Statement</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LC number found anywhere in the statement description (group 1 = the LC). An optional B01/B02 (import bill) or G01/G02 (shipping guarantee) suffix and a trailing dot are not part of it. When a suffix exists the full reference goes to BANK_DC_NO and is used to match the advice (OUR REF NO / USER REF NO)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E72"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Account_Number</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>200153006</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>CITI statement account number -&gt; unit initials written to BATCH_NAME (Bank_Statement CITI branch); an LC lookup can overwrite it</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>200153014</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CITI statement account number -&gt; unit initials written to BATCH_NAME (Bank_Statement CITI branch); an LC lookup can overwrite it</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>1200153029</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CITI statement account number -&gt; unit initials written to BATCH_NAME (Bank_Statement CITI branch); an LC lookup can overwrite it</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CGL</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>200386019</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CITI statement account number -&gt; unit initials written to BATCH_NAME (Bank_Statement CITI branch); an LC lookup can overwrite it</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CGL</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>200386027</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>CITI statement account number -&gt; unit initials written to BATCH_NAME (Bank_Statement CITI branch); an LC lookup can overwrite it</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CGL</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>1200386015</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CITI statement account number -&gt; unit initials written to BATCH_NAME (Bank_Statement CITI branch); an LC lookup can overwrite it</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GFL</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>200837002</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CITI statement account number -&gt; unit initials written to BATCH_NAME (Bank_Statement CITI branch); an LC lookup can overwrite it</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GFL</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>200837029</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CITI statement account number -&gt; unit initials written to BATCH_NAME (Bank_Statement CITI branch); an LC lookup can overwrite it</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GFL</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>1200837009</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CITI statement account number -&gt; unit initials written to BATCH_NAME (Bank_Statement CITI branch); an LC lookup can overwrite it</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CWPL</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>200897005</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CITI statement account number -&gt; unit initials written to BATCH_NAME (Bank_Statement CITI branch); an LC lookup can overwrite it</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CWPL</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>200897013</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>CITI statement account number -&gt; unit initials written to BATCH_NAME (Bank_Statement CITI branch); an LC lookup can overwrite it</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CWPL</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>200897021</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CITI statement account number -&gt; unit initials written to BATCH_NAME (Bank_Statement CITI branch); an LC lookup can overwrite it</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5075,7 +5347,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29.6328125" customWidth="1" min="1" max="1"/>
@@ -5131,6 +5403,21 @@
           <t>Output_Sheet</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Advice_Required</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>LC_Required</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Account_Section</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5154,6 +5441,21 @@
       <c r="F2" t="n">
         <v>27201020010</v>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5177,6 +5479,21 @@
       <c r="F3" t="n">
         <v>27201020010</v>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5200,6 +5517,21 @@
       <c r="F4" t="n">
         <v>27201020010</v>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5220,6 +5552,21 @@
       <c r="D5" t="n">
         <v>45101010013</v>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5248,6 +5595,21 @@
       <c r="F6" t="n">
         <v>41101096008</v>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5276,6 +5638,21 @@
       <c r="F7" t="n">
         <v>41101096008</v>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5296,6 +5673,21 @@
       <c r="D8" t="n">
         <v>45101010013</v>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5316,6 +5708,21 @@
       <c r="D9" t="n">
         <v>45101010013</v>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5336,6 +5743,21 @@
       <c r="D10" t="n">
         <v>45101010013</v>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5356,6 +5778,21 @@
       <c r="D11" t="n">
         <v>45101010013</v>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5376,6 +5813,21 @@
       <c r="D12" t="n">
         <v>45101010014</v>
       </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5396,6 +5848,21 @@
       <c r="D13" t="n">
         <v>45101010014</v>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5416,6 +5883,21 @@
       <c r="D14" t="n">
         <v>45101010014</v>
       </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5476,6 +5958,21 @@
       <c r="D17" t="n">
         <v>45101010004</v>
       </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5496,6 +5993,21 @@
       <c r="D18" t="n">
         <v>45101010004</v>
       </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5516,6 +6028,21 @@
       <c r="D19" t="n">
         <v>45101010004</v>
       </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5536,6 +6063,21 @@
       <c r="D20" t="n">
         <v>45101010004</v>
       </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5556,6 +6098,21 @@
       <c r="D21" t="n">
         <v>45101010004</v>
       </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5576,6 +6133,21 @@
       <c r="D22" t="n">
         <v>45101010004</v>
       </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5596,6 +6168,21 @@
       <c r="D23" t="n">
         <v>45101010004</v>
       </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5636,6 +6223,21 @@
       <c r="D25" t="n">
         <v>45101010004</v>
       </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>BDT=No|USD=Yes</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>BDT=No|USD=Must</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>CD|ERQ</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5658,7 +6260,22 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>TT@USD|TT@EUR</t>
+          <t>EUR@EUR|GRN@USD</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>ERQ</t>
         </is>
       </c>
     </row>
@@ -5737,6 +6354,21 @@
           <t>45101010004</t>
         </is>
       </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5759,6 +6391,21 @@
           <t>45101010004</t>
         </is>
       </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5781,6 +6428,21 @@
           <t>45101010005</t>
         </is>
       </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5818,6 +6480,21 @@
           <t>MACHINERY@EUR|GRN@USD</t>
         </is>
       </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>ERQ</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5860,6 +6537,356 @@
       <c r="I34" t="inlineStr">
         <is>
           <t>MACHINERY@EUR|GRN@USD</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>SUNDRY</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Interest ON STL</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Short Term Loan</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>45101010002</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>STL Payment</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Short Term Loan</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>27401010002</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Interest ON LTL</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Long Term Loan</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>45101010001</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>LTL Payment</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Long Term Loan</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>24201010001</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>STL Received</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Short Term Loan</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Debit Memo</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>27401010002</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>LTL Received</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Long Term Loan</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>24201010001</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ORM TAX (WITHHOLDING)</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>WITHOLDING TAX</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>NEEDS DECISION: Citi NA: Need to Discuss - tax on foreign salary / service payment</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>CD|ERQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>OUTGOING RTGS TRANSFER (SALARY)</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>OUTGOING RTGS TRANSFER</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>NEEDS DECISION: Citi NA: Need to Discuss - salary / inland payment</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>CD|ERQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>FT OUTGOING - SWIFT</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>FT OUTGOING - SWIFT</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>NEEDS DECISION: Citi NA: Need to Discuss - foreign payment</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>CD|ERQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>UPAS Liabilitiy</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>UPAS Liabilitie</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>NEEDS DECISION: Citi NA says not automated - knock to bank then forward MS Excel advice; only payment invoice already prepared</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>SUNDRY</t>
         </is>
       </c>
     </row>
@@ -9370,7 +10397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9419,6 +10446,21 @@
           <t>Output_Sheet</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Advice_Required</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>LC_Required</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Account_Section</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9446,6 +10488,21 @@
           <t>27201020010</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9473,6 +10530,21 @@
           <t>27201020010</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9500,6 +10572,21 @@
           <t>27201020010</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9527,11 +10614,26 @@
           <t>27201020010</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>APPLICATION CHARGE AGAINST</t>
+          <t>COURIER CHARGE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -9547,13 +10649,28 @@
       <c r="D6" t="inlineStr">
         <is>
           <t>45101010013</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TT CHG AGAINST FUND</t>
+          <t>Shipping guarantee issuance charge</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -9569,13 +10686,28 @@
       <c r="D7" t="inlineStr">
         <is>
           <t>45101010013</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SWIFT CHG AGAINST FUND</t>
+          <t>Certificate charge</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -9591,13 +10723,28 @@
       <c r="D8" t="inlineStr">
         <is>
           <t>45101010013</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>COURIER CHARGE</t>
+          <t>Credit Report Charge</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9613,13 +10760,28 @@
       <c r="D9" t="inlineStr">
         <is>
           <t>45101010013</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Shipping guarantee issuance charge</t>
+          <t>IMPORT BILL RETIREMENT</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -9634,14 +10796,39 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>45101010013:41101096008</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>45101010013</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>41101096008</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Certificate charge</t>
+          <t>SG ISSUANCE CHARGE</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -9656,19 +10843,44 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>45101010013:41101096008</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>45101010013</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>41101096008</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Credit Report Charge</t>
+          <t>LC STAMP CHARGE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>OTHER CHARGES</t>
+          <t>LC OPENING CHAR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -9678,19 +10890,44 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>45101010013</t>
+          <t>15303010001:27201020010</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>15303010001</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>27201020010</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>IMPORT BILL RETIREMENT</t>
+          <t>LC ISSUE SWIFT CHG</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>OTHER CHARGES</t>
+          <t>LC OPENING CHAR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -9700,29 +10937,44 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>45101010013:41101096008</t>
+          <t>15303010001:27201020010</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>45101010013</t>
+          <t>15303010001</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>41101096008</t>
+          <t>27201020010</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SG ISSUANCE CHARGE</t>
+          <t>LC AMND SWIFT CHG</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>OTHER CHARGES</t>
+          <t>LC OPENING CHAR</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -9732,24 +10984,39 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>45101010013:41101096008</t>
+          <t>15303010001:27201020010</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>45101010013</t>
+          <t>15303010001</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>41101096008</t>
+          <t>27201020010</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LC STAMP CHARGE</t>
+          <t>CHARGE FOR CNF CERTIFICATE</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -9764,24 +11031,29 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>45101010013:41101096008</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>45101010013</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>41101096008</t>
+          <t>45101010004</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LC ISSUE SWIFT CHG</t>
+          <t>CHARGE FOR NOC CERTIFICATE</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -9796,24 +11068,29 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>45101010013:41101096008</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>45101010013</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>41101096008</t>
+          <t>45101010004</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LC AMND SWIFT CHG</t>
+          <t>CHARGE FOR FOC CERTIFICATE</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -9828,24 +11105,29 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>45101010013:41101096008</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>45101010013</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>41101096008</t>
+          <t>45101010004</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CHARGE FOR CNF CERTIFICATE</t>
+          <t>CHARGE FOR BL</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -9861,13 +11143,28 @@
       <c r="D18" t="inlineStr">
         <is>
           <t>45101010004</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CHARGE FOR NOC CERTIFICATE</t>
+          <t>CHARGES FOR BL ENDORSE</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -9883,13 +11180,28 @@
       <c r="D19" t="inlineStr">
         <is>
           <t>45101010004</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CHARGE FOR FOC CERTIFICATE</t>
+          <t>PROCESSING FEE</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -9905,13 +11217,28 @@
       <c r="D20" t="inlineStr">
         <is>
           <t>45101010004</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CHARGE FOR BL</t>
+          <t>EXCISE DUTY</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -9927,13 +11254,28 @@
       <c r="D21" t="inlineStr">
         <is>
           <t>45101010004</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CHARGES FOR BL ENDORSE</t>
+          <t>BANKERS CHEQUE ISSUANCE COMMISSION</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -9949,13 +11291,28 @@
       <c r="D22" t="inlineStr">
         <is>
           <t>45101010004</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PROCESSING FEE</t>
+          <t>VAT on BANKERS CHEQUE ISSUANCE COMMISSION</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -9971,13 +11328,28 @@
       <c r="D23" t="inlineStr">
         <is>
           <t>45101010004</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EXCISE DUTY</t>
+          <t>RJSC Search Report</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -9993,13 +11365,28 @@
       <c r="D24" t="inlineStr">
         <is>
           <t>45101010004</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>BANKERS CHEQUE ISSUANCE COMMISSION</t>
+          <t>BG DBLBG20262250400 BG  CASH COLLATERAL</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -10007,21 +11394,31 @@
           <t>OTHER CHARGES</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>45101010004</t>
+          <t>15302020004</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>VAT on BANKERS CHEQUE ISSUANCE COMMISSION</t>
+          <t>BG DBLBG20262250400 STAMP CHARGE REALIZE</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -10029,21 +11426,31 @@
           <t>OTHER CHARGES</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>45101010004</t>
+          <t>45101010013</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>RJSC Search Report</t>
+          <t>BG DBLBG20262250400 ISSUE COMMISSION</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -10051,21 +11458,31 @@
           <t>OTHER CHARGES</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>45101010004</t>
+          <t>45101010013</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BG DBLBG20262250400 BG  CASH COLLATERAL</t>
+          <t>BG DBLBG20262250400 VAT - BG COMMISION.</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -10075,14 +11492,29 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>15302020004</t>
+          <t>45101010013</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BG DBLBG20262250400 STAMP CHARGE REALIZE</t>
+          <t>BG Refund DBLBG20252252086 BG CASH COLLATERAL</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -10092,14 +11524,29 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>45101010013</t>
+          <t>15302020004</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BG DBLBG20262250400 ISSUE COMMISSION</t>
+          <t>EXP CERTIFICATION</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -10109,14 +11556,29 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>45101010013</t>
+          <t>45101010014</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BG DBLBG20262250400 VAT - BG COMMISION.</t>
+          <t>MISCELLANEOUS CHARGE</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -10126,14 +11588,29 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>45101010013</t>
+          <t>45101010014</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BG Refund DBLBG20252252086 BG CASH COLLATERAL</t>
+          <t>EB COLLECTION CHARGE</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -10143,31 +11620,46 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>15302020004</t>
+          <t>45101010014</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>EXP CERTIFICATION</t>
+          <t>IMPORT BILL LIQUIDATION</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>OTHER CHARGES</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>45101010014</t>
+          <t>Bills Payable</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>DFC</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>MISCELLANEOUS CHARGE</t>
+          <t>FDD CHARGE</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -10175,16 +11667,36 @@
           <t>OTHER CHARGES</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>45101010014</t>
+          <t>45101010013</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>DFC</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>EB COLLECTION CHARGE</t>
+          <t>TT ISSUE COMMISSION</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -10192,21 +11704,46 @@
           <t>OTHER CHARGES</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>45101010014</t>
+          <t>45101010013</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>TT@USD|TT@EUR</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Interrest on OD</t>
+          <t>Interest on EDF</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>OTHER CHARGES</t>
+          <t>EDF Liabilities</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -10216,19 +11753,39 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>45101010005</t>
+          <t>45101010010</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>MACHINERY@EUR|GRN@USD</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>DFC</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Interest ON STL</t>
+          <t>DEBIT INTEREST</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Short Term Loan</t>
+          <t>OTHER CHARGES</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -10238,283 +11795,140 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>45101010002</t>
+          <t>45101010005</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Interest ON LTL</t>
+          <t>corresponding bank charge</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Long Term Loan</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>45101010001</t>
+          <t>OTHER CHARGES</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>ERQ</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>STL Payment</t>
+          <t>EDF Liabilities</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Short Term Loan</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>27401010002</t>
+          <t>EDF Liabilities</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>DFC</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LTL Payment</t>
+          <t>Commission, SWIFT TT [Service]</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Long Term Loan</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>24201010001</t>
+          <t>OTHER CHARGES</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>STL Received</t>
+          <t>TT Goods related</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Short Term Loan</t>
+          <t>Accessories/Fabrics/Spare Pars</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Debit Memo</t>
+          <t>Prepayment</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>27401010002</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>LTL Received</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Long Term Loan</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Debit Memo</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>24201010001</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>IMPORT BILL LIQUIDATION</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Bills Payable</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>FDD CHARGE</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Bills Payable</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>45101010013</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>TT ISSUE COMMISSION</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>OTHER CHARGES</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>45101010013</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
+          <t>15303010001</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>OUTWARD PAY|TT GOODS</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
         <is>
           <t>TT@USD|TT@EUR</t>
         </is>
       </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Interest on EDF</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>EDF Liabilities</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>45101010010</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>MACHINERY@EUR|GRN@USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>DEBIT INTEREST</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>OTHER CHARGES</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>45101010005</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>corresponding bank charge</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>OTHER CHARGES</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>EDF Liabilities</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>EDF Liabilities</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>OUTWARD PAYMNET</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Accessories/Fabrics/Spare Pars</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Prepayment</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>15303010001</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>OUTWARD PAY|TT GOODS</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>TT@USD|TT@EUR</t>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>ERQ</t>
         </is>
       </c>
     </row>
@@ -12569,7 +13983,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Rules sheet ready (advice layout keys); TT / GRN / Machinery advice rules are TBD</t>
+          <t>Rules sheet ready; unit accounts in CITI_Units; routing PRINCIPAL -&gt; TT or Machinery (EUR bill also fills EUR columns); machinery interest split is a later module</t>
         </is>
       </c>
     </row>
@@ -12648,7 +14062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14048,7 +15462,7 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>TT_Amount|TT_Amount_Expense_Type|TT_Account|TT_INVOICE_NO|TT_DESCRIPTION|TT_Invoice_Voucher_No|TT_Payment_Number|TT_Clear_Transaction|COMMISION_TT|COMMISION_TT_Expense_Type|COMMISION_TT_Acount|COMMISION_TT_INVOICE_NO|COMMISION_TT_DESCRIPTION|COMMISION_TT_Invoice_Voucher_No|COMMISION_TT_Payment_Number|COMMISION_TT_Clear_Transaction</t>
+          <t>TT_Amount|TT_Amount_Expense_Type|TT_Account</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -14075,7 +15489,7 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>GRN_NUMBER|REMITTED_AMOUNT|INT_AMOUNT|Match_Invoice_No</t>
+          <t>GRN_NUMBER|REMITTED_AMOUNT|INT_AMOUNT|EXCISE_AMOUNT|Match_Invoice_No</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -14507,7 +15921,7 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>LC ISSUANCE COMMISSION=&gt;LC ISSUANCE COMMISSION|LC AMENDMENT COMMISSION=&gt;LC AMENDMENT COMMISSION|ACCEPTANCE COMMISSION=&gt;ACCEPTANCE COMMISSION CHARGE</t>
+          <t>LC ISSUANCE COMMISSION=&gt;LC ISSUANCE COMMISSION|LC AMENDMENT COMMISSION=&gt;LC AMENDMENT COMMISSION|ACCEPTANCE COMMISSION=&gt;ACCEPTANCE COMMISSION CHARGE|PRINCIPAL LIQUIDATION=&gt;PRINCIPAL LIQUIDATION</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -14532,7 +15946,11 @@
           <t>LC_Number_Regex</t>
         </is>
       </c>
-      <c r="C70" s="4" t="n"/>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>^5\d{9}$</t>
+        </is>
+      </c>
       <c r="D70" t="inlineStr">
         <is>
           <t>later</t>
@@ -14823,7 +16241,7 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -14850,7 +16268,7 @@
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -14861,6 +16279,411 @@
       <c r="E82" t="inlineStr">
         <is>
           <t>Days after the statement date searched for the advice mail (0 = same day). Not used by SCB</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>ADVICE_TEXT</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Adv_LC_Regex</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>(?:LC NO\s*:|LC REF)\s*([0-9A-Za-z\-]+)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>CITI advice reader</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LC number on the CITI advice: "LC NO : 5634610197" or "... LC REF 5634611205" in OTHER INSTRUCTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>ADVICE_TEXT</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Adv_Principal_Regex</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>PRINCIPAL LIQUIDATION[^\r\n]*?[A-Z]{3}\s*([\d,]+\.\d+)(?=\s*(?:\r|\n|$))</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>CITI advice reader</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Principal amount (debited currency) on the REPRESENTING block</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>ADVICE_TEXT</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Adv_Interest_Regex</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>INTEREST OF[^\r\n]*?[A-Z]{3}\s*([\d,]+\.\d+)(?=\s*(?:\r|\n|$))</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>CITI advice reader</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Interest amount (debited currency) on the REPRESENTING block</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>ADVICE_TEXT</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Adv_Excise_Regex</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>EXCISE DUTY OF[^\r\n]*?[A-Z]{3}\s*([\d,]+\.\d+)(?=\s*(?:\r|\n|$))</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>CITI advice reader</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Excise duty amount (debited currency) on the REPRESENTING block</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>OUTPUT_COLUMNS</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Rename_INT_AMOUNT</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Interest</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Advice_pdf</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>CITI only: header shown in the output for INT_AMOUNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>OUTPUT_COLUMNS</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Rename_EXCISE_AMOUNT</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Excise Duty</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Advice_pdf</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>CITI only: header shown in the output for EXCISE_AMOUNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>ADVICE_TEXT</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Adv_Block_Start</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>REPRESENTING</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>CITI_advice_reader</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Text that starts the charge block of the advice</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>ADVICE_TEXT</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Adv_Block_End</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>TOTAL AMOUNT DEBITED</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>CITI_advice_reader</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Text that ends the charge block of the advice</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>ADVICE_TEXT</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Adv_Inline_Amount_Regex</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>[A-Z]{3}\s*([\d,]+\.\d+)\s*$</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>CITI_advice_reader</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Amount at the end of a label line, e.g. INTEREST OF USD146.20</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>ADVICE_TEXT</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Adv_Alone_Amount_Regex</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>^[A-Z]{3}\s*([\d,]+\.\d+)$</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>CITI_advice_reader</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Amount alone on a line, listed after the labels (read in label order)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>ADVICE_TEXT</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Adv_Principal_Label</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>PRINCIPAL LIQUIDATION</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>CITI_advice_reader</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Advice line label for the principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ADVICE_TEXT</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Adv_Interest_Label</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>INTEREST OF</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>CITI_advice_reader</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Advice line label for the interest</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>ADVICE_TEXT</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Adv_Excise_Label</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>EXCISE DUTY OF</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>CITI_advice_reader</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Advice line label for the excise duty</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>EVENTS</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Skip_Marker</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>NEEDS DECISION</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>CITI_advice_reader</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Text in the CITI sheet Review column that makes the reader skip the event</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>CURRENCY</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Eur_Bill_Currency</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>CITI_advice_reader</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Bill currency that also fills the EUR columns</t>
         </is>
       </c>
     </row>

</xml_diff>